<commit_message>
📊 Actualización automática de estadísticas
</commit_message>
<xml_diff>
--- a/estadisticas.xlsx
+++ b/estadisticas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estadisticas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Estadisticas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,58 +413,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tema</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>pregunta_corta</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pregunta_completa</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>intentos</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>aciertos</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>fallos</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>pct_fallos</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>pct_aciertos</t>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>porcentaje_fallos</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>porcentaje_aciertos</t>
         </is>
       </c>
     </row>
@@ -2589,6 +2567,38 @@
         <v>0</v>
       </c>
       <c r="H67" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>B Completo revistas</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>20. La mejor forma de recuperarse de la fatiga cua</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>20. La mejor forma de recuperarse de la fatiga cuando se conduce, es...</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>